<commit_message>
fix stale yield labels in Excel sheet titles (values were already correct)
</commit_message>
<xml_diff>
--- a/assets/LCOH_Model_Kuhyar_Saeedi.xlsx
+++ b/assets/LCOH_Model_Kuhyar_Saeedi.xlsx
@@ -339,7 +339,7 @@
     <t xml:space="preserve">Excluded (paper: 1644)</t>
   </si>
   <si>
-    <t xml:space="preserve">MODEL — South Italy (Naples), yield 1272 kWh/kWp/yr</t>
+    <t xml:space="preserve">MODEL — South Italy (Naples), yield 1497 kWh/kWp/yr (PVGIS-SARAH3)</t>
   </si>
   <si>
     <t xml:space="preserve">12 configurations — all values live-linked to Parameters sheet</t>
@@ -474,7 +474,7 @@
     <t xml:space="preserve">Medium_LG</t>
   </si>
   <si>
-    <t xml:space="preserve">MODEL — North Italy (Milan), yield 1050 kWh/kWp/yr</t>
+    <t xml:space="preserve">MODEL — North Italy (Milan), yield 1369 kWh/kWp/yr (PVGIS-SARAH3)</t>
   </si>
   <si>
     <t xml:space="preserve">LCOH RESULTS SUMMARY (€/kg H2)</t>
@@ -795,111 +795,111 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>